<commit_message>
revamp the Theres du mois workflow improve OneShot and made it public visible
</commit_message>
<xml_diff>
--- a/TempsDeTravail.xlsx
+++ b/TempsDeTravail.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\ClubPhoto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFED59A4-4CB6-49A0-960E-41B0B1E5AD75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56CDB339-0CD6-4AA8-B3F9-B29D29D51565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{29D00352-7DCC-4914-AE3D-35C4116899F6}"/>
   </bookViews>
@@ -438,11 +438,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{963FE1CA-F18E-4BB6-AE80-3CF535E7A177}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.08984375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.6328125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="17.453125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7265625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.35">
@@ -461,6 +461,14 @@
         <v>10.006944444444445</v>
       </c>
     </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1">
+        <v>46185</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2.4305555555555556E-3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
align de x of delete comment with at the level of the name of who did the comment
</commit_message>
<xml_diff>
--- a/TempsDeTravail.xlsx
+++ b/TempsDeTravail.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\ClubPhoto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56CDB339-0CD6-4AA8-B3F9-B29D29D51565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD106AA7-DAA8-4B5D-83CB-13DB5B430A39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{29D00352-7DCC-4914-AE3D-35C4116899F6}"/>
+    <workbookView xWindow="5780" yWindow="3580" windowWidth="28800" windowHeight="15370" xr2:uid="{29D00352-7DCC-4914-AE3D-35C4116899F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -438,7 +438,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{963FE1CA-F18E-4BB6-AE80-3CF535E7A177}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.453125" style="1" customWidth="1"/>
@@ -466,7 +466,15 @@
         <v>46185</v>
       </c>
       <c r="B3" s="2">
-        <v>2.4305555555555556E-3</v>
+        <v>5.5555555555555558E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="1">
+        <v>46186</v>
+      </c>
+      <c r="B4" s="2">
+        <v>2.0833333333333333E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>